<commit_message>
Delivery of feedback from Emily on 18-09-2026
</commit_message>
<xml_diff>
--- a/docs/Import/Revitalise-WBS-Grant-Automation-v0.6.xlsx
+++ b/docs/Import/Revitalise-WBS-Grant-Automation-v0.6.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10830"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10917"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://argelisconsultancy.sharepoint.com/teams/RevitaliseRespiteHolidays/Gedeelde documenten/Optimisation Grant Application Process/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://argelisconsultancy.sharepoint.com/teams/RevitaliseRespiteHolidays/Gedeelde documenten/Optimisation Grant Application Process/Repository/Revitalise/docs/Import/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="3" documentId="8_{DAD0A581-B05E-AB43-A41A-21FEB48A0E94}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0C930A91-3DD3-BC40-8163-363DE837814C}"/>
+  <xr:revisionPtr revIDLastSave="6" documentId="8_{DAD0A581-B05E-AB43-A41A-21FEB48A0E94}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{190209BA-EC7B-434E-8466-54FE2526ACBC}"/>
   <bookViews>
-    <workbookView xWindow="4740" yWindow="1260" windowWidth="39180" windowHeight="23520" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="780" windowWidth="36000" windowHeight="21480" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Summary" sheetId="1" r:id="rId1"/>
@@ -2736,132 +2736,136 @@
       </c>
     </row>
     <row r="26" spans="1:11" ht="24.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A26" s="6" t="s">
+      <c r="A26" s="9" t="s">
         <v>124</v>
       </c>
-      <c r="B26" s="6" t="s">
+      <c r="B26" s="9" t="s">
         <v>125</v>
       </c>
-      <c r="C26" s="6" t="s">
+      <c r="C26" s="9" t="s">
         <v>126</v>
       </c>
-      <c r="D26" s="6" t="s">
+      <c r="D26" s="9" t="s">
         <v>127</v>
       </c>
-      <c r="E26" s="6" t="s">
+      <c r="E26" s="9" t="s">
         <v>128</v>
       </c>
-      <c r="F26" s="6">
+      <c r="F26" s="9">
         <v>4</v>
       </c>
-      <c r="G26" s="6">
+      <c r="G26" s="9">
         <v>6</v>
       </c>
-      <c r="H26" s="6" t="s">
+      <c r="H26" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="I26" s="6" t="s">
+      <c r="I26" s="9" t="s">
         <v>66</v>
       </c>
-      <c r="J26" s="6" t="s">
+      <c r="J26" s="9" t="s">
         <v>129</v>
       </c>
+      <c r="K26" s="13"/>
     </row>
     <row r="27" spans="1:11" ht="36" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A27" s="6" t="s">
+      <c r="A27" s="9" t="s">
         <v>130</v>
       </c>
-      <c r="B27" s="6" t="s">
+      <c r="B27" s="9" t="s">
         <v>125</v>
       </c>
-      <c r="C27" s="6" t="s">
+      <c r="C27" s="9" t="s">
         <v>126</v>
       </c>
-      <c r="D27" s="6" t="s">
+      <c r="D27" s="9" t="s">
         <v>131</v>
       </c>
-      <c r="E27" s="6" t="s">
+      <c r="E27" s="9" t="s">
         <v>132</v>
       </c>
-      <c r="F27" s="6">
+      <c r="F27" s="9">
         <v>4</v>
       </c>
-      <c r="G27" s="6">
+      <c r="G27" s="9">
         <v>6</v>
       </c>
-      <c r="H27" s="6" t="s">
+      <c r="H27" s="9" t="s">
         <v>124</v>
       </c>
-      <c r="I27" s="6" t="s">
+      <c r="I27" s="9" t="s">
         <v>66</v>
       </c>
-      <c r="J27" s="6" t="s">
+      <c r="J27" s="9" t="s">
         <v>102</v>
       </c>
+      <c r="K27" s="13"/>
     </row>
     <row r="28" spans="1:11" ht="24.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A28" s="6" t="s">
+      <c r="A28" s="9" t="s">
         <v>133</v>
       </c>
-      <c r="B28" s="6" t="s">
+      <c r="B28" s="9" t="s">
         <v>125</v>
       </c>
-      <c r="C28" s="6" t="s">
+      <c r="C28" s="9" t="s">
         <v>126</v>
       </c>
-      <c r="D28" s="6" t="s">
+      <c r="D28" s="9" t="s">
         <v>134</v>
       </c>
-      <c r="E28" s="6" t="s">
+      <c r="E28" s="9" t="s">
         <v>135</v>
       </c>
-      <c r="F28" s="6">
+      <c r="F28" s="9">
         <v>2</v>
       </c>
-      <c r="G28" s="6">
+      <c r="G28" s="9">
         <v>3</v>
       </c>
-      <c r="H28" s="6" t="s">
+      <c r="H28" s="9" t="s">
         <v>130</v>
       </c>
-      <c r="I28" s="6" t="s">
+      <c r="I28" s="9" t="s">
         <v>66</v>
       </c>
-      <c r="J28" s="6" t="s">
+      <c r="J28" s="9" t="s">
         <v>136</v>
       </c>
+      <c r="K28" s="13"/>
     </row>
     <row r="29" spans="1:11" ht="24.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A29" s="6" t="s">
+      <c r="A29" s="9" t="s">
         <v>137</v>
       </c>
-      <c r="B29" s="6" t="s">
+      <c r="B29" s="9" t="s">
         <v>125</v>
       </c>
-      <c r="C29" s="6" t="s">
+      <c r="C29" s="9" t="s">
         <v>126</v>
       </c>
-      <c r="D29" s="6" t="s">
+      <c r="D29" s="9" t="s">
         <v>138</v>
       </c>
-      <c r="E29" s="6" t="s">
+      <c r="E29" s="9" t="s">
         <v>139</v>
       </c>
-      <c r="F29" s="6">
+      <c r="F29" s="9">
         <v>3</v>
       </c>
-      <c r="G29" s="6">
+      <c r="G29" s="9">
         <v>4</v>
       </c>
-      <c r="H29" s="6" t="s">
+      <c r="H29" s="9" t="s">
         <v>130</v>
       </c>
-      <c r="I29" s="6" t="s">
+      <c r="I29" s="9" t="s">
         <v>66</v>
       </c>
-      <c r="J29" s="6" t="s">
+      <c r="J29" s="9" t="s">
         <v>140</v>
       </c>
+      <c r="K29" s="13"/>
     </row>
     <row r="30" spans="1:11" ht="24.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="6" t="s">
@@ -3356,258 +3360,258 @@
       </c>
     </row>
     <row r="45" spans="1:11" ht="24.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A45" s="6" t="s">
+      <c r="A45" s="9" t="s">
         <v>203</v>
       </c>
-      <c r="B45" s="6" t="s">
+      <c r="B45" s="9" t="s">
         <v>204</v>
       </c>
-      <c r="C45" s="6" t="s">
+      <c r="C45" s="9" t="s">
         <v>205</v>
       </c>
-      <c r="D45" s="6" t="s">
+      <c r="D45" s="9" t="s">
         <v>206</v>
       </c>
-      <c r="E45" s="6" t="s">
+      <c r="E45" s="9" t="s">
         <v>207</v>
       </c>
-      <c r="F45" s="6">
+      <c r="F45" s="9">
         <v>4</v>
       </c>
-      <c r="G45" s="6">
+      <c r="G45" s="9">
         <v>6</v>
       </c>
-      <c r="H45" s="6" t="s">
+      <c r="H45" s="9" t="s">
         <v>186</v>
       </c>
-      <c r="I45" s="6" t="s">
+      <c r="I45" s="9" t="s">
         <v>180</v>
       </c>
-      <c r="J45" s="6" t="s">
+      <c r="J45" s="9" t="s">
         <v>208</v>
       </c>
     </row>
     <row r="46" spans="1:11" ht="36" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A46" s="6" t="s">
+      <c r="A46" s="9" t="s">
         <v>209</v>
       </c>
-      <c r="B46" s="6" t="s">
+      <c r="B46" s="9" t="s">
         <v>204</v>
       </c>
-      <c r="C46" s="6" t="s">
+      <c r="C46" s="9" t="s">
         <v>205</v>
       </c>
-      <c r="D46" s="6" t="s">
+      <c r="D46" s="9" t="s">
         <v>210</v>
       </c>
-      <c r="E46" s="6" t="s">
+      <c r="E46" s="9" t="s">
         <v>211</v>
       </c>
-      <c r="F46" s="6">
+      <c r="F46" s="9">
         <v>3</v>
       </c>
-      <c r="G46" s="6">
+      <c r="G46" s="9">
         <v>5</v>
       </c>
-      <c r="H46" s="6" t="s">
+      <c r="H46" s="9" t="s">
         <v>203</v>
       </c>
-      <c r="I46" s="6" t="s">
+      <c r="I46" s="9" t="s">
         <v>180</v>
       </c>
-      <c r="J46" s="6" t="s">
+      <c r="J46" s="9" t="s">
         <v>212</v>
       </c>
     </row>
     <row r="47" spans="1:11" ht="36" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A47" s="6" t="s">
+      <c r="A47" s="9" t="s">
         <v>213</v>
       </c>
-      <c r="B47" s="6" t="s">
+      <c r="B47" s="9" t="s">
         <v>204</v>
       </c>
-      <c r="C47" s="6" t="s">
+      <c r="C47" s="9" t="s">
         <v>205</v>
       </c>
-      <c r="D47" s="6" t="s">
+      <c r="D47" s="9" t="s">
         <v>214</v>
       </c>
-      <c r="E47" s="6" t="s">
+      <c r="E47" s="9" t="s">
         <v>215</v>
       </c>
-      <c r="F47" s="6">
+      <c r="F47" s="9">
         <v>3</v>
       </c>
-      <c r="G47" s="6">
+      <c r="G47" s="9">
         <v>5</v>
       </c>
-      <c r="H47" s="6" t="s">
+      <c r="H47" s="9" t="s">
         <v>203</v>
       </c>
-      <c r="I47" s="6" t="s">
+      <c r="I47" s="9" t="s">
         <v>180</v>
       </c>
-      <c r="J47" s="6" t="s">
+      <c r="J47" s="9" t="s">
         <v>216</v>
       </c>
     </row>
     <row r="48" spans="1:11" ht="36" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A48" s="6" t="s">
+      <c r="A48" s="9" t="s">
         <v>217</v>
       </c>
-      <c r="B48" s="6" t="s">
+      <c r="B48" s="9" t="s">
         <v>204</v>
       </c>
-      <c r="C48" s="6" t="s">
+      <c r="C48" s="9" t="s">
         <v>205</v>
       </c>
-      <c r="D48" s="6" t="s">
+      <c r="D48" s="9" t="s">
         <v>218</v>
       </c>
-      <c r="E48" s="6" t="s">
+      <c r="E48" s="9" t="s">
         <v>219</v>
       </c>
-      <c r="F48" s="6">
+      <c r="F48" s="9">
         <v>3</v>
       </c>
-      <c r="G48" s="6">
+      <c r="G48" s="9">
         <v>5</v>
       </c>
-      <c r="H48" s="6" t="s">
+      <c r="H48" s="9" t="s">
         <v>209</v>
       </c>
-      <c r="I48" s="6" t="s">
+      <c r="I48" s="9" t="s">
         <v>180</v>
       </c>
-      <c r="J48" s="6" t="s">
+      <c r="J48" s="9" t="s">
         <v>220</v>
       </c>
     </row>
     <row r="49" spans="1:10" ht="36" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A49" s="6" t="s">
+      <c r="A49" s="9" t="s">
         <v>221</v>
       </c>
-      <c r="B49" s="6" t="s">
+      <c r="B49" s="9" t="s">
         <v>204</v>
       </c>
-      <c r="C49" s="6" t="s">
+      <c r="C49" s="9" t="s">
         <v>205</v>
       </c>
-      <c r="D49" s="6" t="s">
+      <c r="D49" s="9" t="s">
         <v>222</v>
       </c>
-      <c r="E49" s="6" t="s">
+      <c r="E49" s="9" t="s">
         <v>223</v>
       </c>
-      <c r="F49" s="6">
+      <c r="F49" s="9">
         <v>2</v>
       </c>
-      <c r="G49" s="6">
+      <c r="G49" s="9">
         <v>3</v>
       </c>
-      <c r="H49" s="6" t="s">
+      <c r="H49" s="9" t="s">
         <v>224</v>
       </c>
-      <c r="I49" s="6" t="s">
+      <c r="I49" s="9" t="s">
         <v>180</v>
       </c>
-      <c r="J49" s="6" t="s">
+      <c r="J49" s="9" t="s">
         <v>225</v>
       </c>
     </row>
     <row r="50" spans="1:10" ht="24.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A50" s="6" t="s">
+      <c r="A50" s="9" t="s">
         <v>226</v>
       </c>
-      <c r="B50" s="6" t="s">
+      <c r="B50" s="9" t="s">
         <v>204</v>
       </c>
-      <c r="C50" s="6" t="s">
+      <c r="C50" s="9" t="s">
         <v>205</v>
       </c>
-      <c r="D50" s="6" t="s">
+      <c r="D50" s="9" t="s">
         <v>227</v>
       </c>
-      <c r="E50" s="6" t="s">
+      <c r="E50" s="9" t="s">
         <v>228</v>
       </c>
-      <c r="F50" s="6">
+      <c r="F50" s="9">
         <v>3</v>
       </c>
-      <c r="G50" s="6">
+      <c r="G50" s="9">
         <v>4</v>
       </c>
-      <c r="H50" s="6" t="s">
+      <c r="H50" s="9" t="s">
         <v>229</v>
       </c>
-      <c r="I50" s="6" t="s">
+      <c r="I50" s="9" t="s">
         <v>180</v>
       </c>
-      <c r="J50" s="6" t="s">
+      <c r="J50" s="9" t="s">
         <v>230</v>
       </c>
     </row>
     <row r="51" spans="1:10" ht="36" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A51" s="6" t="s">
+      <c r="A51" s="9" t="s">
         <v>231</v>
       </c>
-      <c r="B51" s="6" t="s">
+      <c r="B51" s="9" t="s">
         <v>204</v>
       </c>
-      <c r="C51" s="6" t="s">
+      <c r="C51" s="9" t="s">
         <v>205</v>
       </c>
-      <c r="D51" s="6" t="s">
+      <c r="D51" s="9" t="s">
         <v>232</v>
       </c>
-      <c r="E51" s="6" t="s">
+      <c r="E51" s="9" t="s">
         <v>233</v>
       </c>
-      <c r="F51" s="6">
+      <c r="F51" s="9">
         <v>2</v>
       </c>
-      <c r="G51" s="6">
+      <c r="G51" s="9">
         <v>3</v>
       </c>
-      <c r="H51" s="6" t="s">
+      <c r="H51" s="9" t="s">
         <v>234</v>
       </c>
-      <c r="I51" s="6" t="s">
+      <c r="I51" s="9" t="s">
         <v>180</v>
       </c>
-      <c r="J51" s="6" t="s">
+      <c r="J51" s="9" t="s">
         <v>115</v>
       </c>
     </row>
     <row r="52" spans="1:10" ht="24.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A52" s="6" t="s">
+      <c r="A52" s="9" t="s">
         <v>235</v>
       </c>
-      <c r="B52" s="6" t="s">
+      <c r="B52" s="9" t="s">
         <v>204</v>
       </c>
-      <c r="C52" s="6" t="s">
+      <c r="C52" s="9" t="s">
         <v>205</v>
       </c>
-      <c r="D52" s="6" t="s">
+      <c r="D52" s="9" t="s">
         <v>117</v>
       </c>
-      <c r="E52" s="6" t="s">
+      <c r="E52" s="9" t="s">
         <v>236</v>
       </c>
-      <c r="F52" s="6">
+      <c r="F52" s="9">
         <v>2</v>
       </c>
-      <c r="G52" s="6">
+      <c r="G52" s="9">
         <v>4</v>
       </c>
-      <c r="H52" s="6" t="s">
+      <c r="H52" s="9" t="s">
         <v>231</v>
       </c>
-      <c r="I52" s="6" t="s">
+      <c r="I52" s="9" t="s">
         <v>180</v>
       </c>
-      <c r="J52" s="6" t="s">
+      <c r="J52" s="9" t="s">
         <v>237</v>
       </c>
     </row>
@@ -3772,98 +3776,98 @@
       </c>
     </row>
     <row r="58" spans="1:10" ht="24.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A58" s="6" t="s">
+      <c r="A58" s="9" t="s">
         <v>261</v>
       </c>
-      <c r="B58" s="6" t="s">
+      <c r="B58" s="9" t="s">
         <v>262</v>
       </c>
-      <c r="C58" s="6" t="s">
+      <c r="C58" s="9" t="s">
         <v>263</v>
       </c>
-      <c r="D58" s="6" t="s">
+      <c r="D58" s="9" t="s">
         <v>264</v>
       </c>
-      <c r="E58" s="6" t="s">
+      <c r="E58" s="9" t="s">
         <v>265</v>
       </c>
-      <c r="F58" s="6">
+      <c r="F58" s="9">
         <v>3</v>
       </c>
-      <c r="G58" s="6">
+      <c r="G58" s="9">
         <v>5</v>
       </c>
-      <c r="H58" s="6" t="s">
+      <c r="H58" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="I58" s="6" t="s">
+      <c r="I58" s="9" t="s">
         <v>243</v>
       </c>
-      <c r="J58" s="6" t="s">
+      <c r="J58" s="9" t="s">
         <v>266</v>
       </c>
     </row>
     <row r="59" spans="1:10" ht="42" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A59" s="6" t="s">
+      <c r="A59" s="9" t="s">
         <v>267</v>
       </c>
-      <c r="B59" s="6" t="s">
+      <c r="B59" s="9" t="s">
         <v>262</v>
       </c>
-      <c r="C59" s="6" t="s">
+      <c r="C59" s="9" t="s">
         <v>263</v>
       </c>
-      <c r="D59" s="6" t="s">
+      <c r="D59" s="9" t="s">
         <v>268</v>
       </c>
-      <c r="E59" s="6" t="s">
+      <c r="E59" s="9" t="s">
         <v>269</v>
       </c>
-      <c r="F59" s="6">
+      <c r="F59" s="9">
         <v>2</v>
       </c>
-      <c r="G59" s="6">
+      <c r="G59" s="9">
         <v>4</v>
       </c>
-      <c r="H59" s="6" t="s">
+      <c r="H59" s="9" t="s">
         <v>32</v>
       </c>
-      <c r="I59" s="6" t="s">
+      <c r="I59" s="9" t="s">
         <v>243</v>
       </c>
-      <c r="J59" s="6" t="s">
+      <c r="J59" s="9" t="s">
         <v>270</v>
       </c>
     </row>
     <row r="60" spans="1:10" ht="28" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A60" s="6" t="s">
+      <c r="A60" s="9" t="s">
         <v>271</v>
       </c>
-      <c r="B60" s="6" t="s">
+      <c r="B60" s="9" t="s">
         <v>262</v>
       </c>
-      <c r="C60" s="6" t="s">
+      <c r="C60" s="9" t="s">
         <v>263</v>
       </c>
-      <c r="D60" s="6" t="s">
+      <c r="D60" s="9" t="s">
         <v>272</v>
       </c>
-      <c r="E60" s="6" t="s">
+      <c r="E60" s="9" t="s">
         <v>273</v>
       </c>
-      <c r="F60" s="6">
+      <c r="F60" s="9">
         <v>4</v>
       </c>
-      <c r="G60" s="6">
+      <c r="G60" s="9">
         <v>6</v>
       </c>
-      <c r="H60" s="6" t="s">
+      <c r="H60" s="9" t="s">
         <v>335</v>
       </c>
-      <c r="I60" s="6" t="s">
+      <c r="I60" s="9" t="s">
         <v>243</v>
       </c>
-      <c r="J60" s="6" t="s">
+      <c r="J60" s="9" t="s">
         <v>274</v>
       </c>
     </row>
@@ -4094,26 +4098,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="f28f5036-0c97-4fb2-9995-e6511ad4535b">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="d3a2e4d4-5189-48ac-a210-e1294fbd99f3" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010019BFD6B84F7029419816FFCF5AF812DE" ma:contentTypeVersion="9" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ae75f7d6110eb3c01e30b5864ecce8d9">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="f28f5036-0c97-4fb2-9995-e6511ad4535b" xmlns:ns3="d3a2e4d4-5189-48ac-a210-e1294fbd99f3" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="5f758225586994ab2ed7147b7dc97d7e" ns2:_="" ns3:_="">
     <xsd:import namespace="f28f5036-0c97-4fb2-9995-e6511ad4535b"/>
@@ -4294,32 +4278,27 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BBC56B45-ED14-43B1-B900-5E16DD26A51C}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="f28f5036-0c97-4fb2-9995-e6511ad4535b">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="d3a2e4d4-5189-48ac-a210-e1294fbd99f3" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D5BE8830-D071-4623-9F55-2E342F354848}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="d3a2e4d4-5189-48ac-a210-e1294fbd99f3"/>
-    <ds:schemaRef ds:uri="f28f5036-0c97-4fb2-9995-e6511ad4535b"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AC477932-3CE1-4CBF-A1AC-2584224523DC}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -4336,4 +4315,29 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D5BE8830-D071-4623-9F55-2E342F354848}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="f28f5036-0c97-4fb2-9995-e6511ad4535b"/>
+    <ds:schemaRef ds:uri="d3a2e4d4-5189-48ac-a210-e1294fbd99f3"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BBC56B45-ED14-43B1-B900-5E16DD26A51C}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Changes as part of the clean-up and recheck of delivered work of previous delivered work.
Calculate & Score flow, added auto-reject calculations.
Finalise decision flow, to send reviews to Grants.
Capture Payment flow, to finalise the payment and the grant.
</commit_message>
<xml_diff>
--- a/docs/Import/Revitalise-WBS-Grant-Automation-v0.6.xlsx
+++ b/docs/Import/Revitalise-WBS-Grant-Automation-v0.6.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10917"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11011"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://argelisconsultancy.sharepoint.com/teams/RevitaliseRespiteHolidays/Gedeelde documenten/Optimisation Grant Application Process/Repository/Revitalise/docs/Import/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="6" documentId="8_{DAD0A581-B05E-AB43-A41A-21FEB48A0E94}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{190209BA-EC7B-434E-8466-54FE2526ACBC}"/>
+  <xr:revisionPtr revIDLastSave="7" documentId="8_{DAD0A581-B05E-AB43-A41A-21FEB48A0E94}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C7970EF7-AAAB-4748-A3F5-2FCEBD1D918E}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="780" windowWidth="36000" windowHeight="21480" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="5200" yWindow="600" windowWidth="41120" windowHeight="23920" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Summary" sheetId="1" r:id="rId1"/>
@@ -3519,7 +3519,7 @@
         <v>225</v>
       </c>
     </row>
-    <row r="50" spans="1:10" ht="24.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:10" ht="42" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A50" s="9" t="s">
         <v>226</v>
       </c>
@@ -4098,6 +4098,26 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="f28f5036-0c97-4fb2-9995-e6511ad4535b">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="d3a2e4d4-5189-48ac-a210-e1294fbd99f3" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010019BFD6B84F7029419816FFCF5AF812DE" ma:contentTypeVersion="9" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ae75f7d6110eb3c01e30b5864ecce8d9">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="f28f5036-0c97-4fb2-9995-e6511ad4535b" xmlns:ns3="d3a2e4d4-5189-48ac-a210-e1294fbd99f3" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="5f758225586994ab2ed7147b7dc97d7e" ns2:_="" ns3:_="">
     <xsd:import namespace="f28f5036-0c97-4fb2-9995-e6511ad4535b"/>
@@ -4278,27 +4298,32 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="f28f5036-0c97-4fb2-9995-e6511ad4535b">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="d3a2e4d4-5189-48ac-a210-e1294fbd99f3" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BBC56B45-ED14-43B1-B900-5E16DD26A51C}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D5BE8830-D071-4623-9F55-2E342F354848}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="f28f5036-0c97-4fb2-9995-e6511ad4535b"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="d3a2e4d4-5189-48ac-a210-e1294fbd99f3"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AC477932-3CE1-4CBF-A1AC-2584224523DC}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -4315,29 +4340,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D5BE8830-D071-4623-9F55-2E342F354848}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="f28f5036-0c97-4fb2-9995-e6511ad4535b"/>
-    <ds:schemaRef ds:uri="d3a2e4d4-5189-48ac-a210-e1294fbd99f3"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BBC56B45-ED14-43B1-B900-5E16DD26A51C}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>